<commit_message>
fix: update vol3 lime profile url
</commit_message>
<xml_diff>
--- a/content/events/vol-3/vol-3_guest_input_template.xlsx
+++ b/content/events/vol-3/vol-3_guest_input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yana/Desktop/VoiceTree/40_web/projects/260221_PICKUPLIVER/content/events/vol-3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65EBC7EC-30A7-864F-9A99-DEC7AF794F62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67BA2BF-0A75-B243-8FDE-00A1AADBEEF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,9 +110,6 @@
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>https://web.colorsing.com/share/live?live_id=deeb30e9-4163-4f35-bb19-17769e3f3b84</t>
-  </si>
-  <si>
     <t>https://web.colorsing.com/share/user?user_id=aca27f9b-0114-455f-98e3-bf81702d7b58</t>
   </si>
   <si>
@@ -148,6 +145,10 @@
     <rPh sb="0" eb="2">
       <t>シノミヤ</t>
     </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>https://web.colorsing.com/share/user?user_id=299afae1-ff3f-4512-9ebd-02d86d0f53eb</t>
     <phoneticPr fontId="3"/>
   </si>
 </sst>
@@ -155,7 +156,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -185,6 +186,14 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -208,17 +217,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -578,7 +590,7 @@
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
@@ -592,10 +604,10 @@
         <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -606,10 +618,10 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" t="s">
         <v>32</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
       </c>
       <c r="E4" t="s">
         <v>26</v>
@@ -623,10 +635,10 @@
         <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
         <v>24</v>
@@ -640,10 +652,10 @@
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -653,11 +665,11 @@
       <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
-        <v>27</v>
+      <c r="C7" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E7" t="s">
         <v>25</v>
@@ -665,6 +677,9 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3"/>
+  <hyperlinks>
+    <hyperlink ref="C7" r:id="rId1" xr:uid="{B38BDEAD-57A0-434A-A64F-F2EF1E90F92F}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>